<commit_message>
Commit author's workbook fixes (Milic, Körtik, Carter 2006)
data1.xlsx / data2.xlsx as saved after the author's Excel cleanup:
- Milic Carpathian rows repaired
- Körtik (Carter et al 2013) Source column merged; negatives/brackets removed
- Carter et al. 2006 re-aligned to start at column A

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/article_tables/data1.xlsx
+++ b/data/article_tables/data1.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492F120B-1C20-4B56-B58A-CC62FCC80D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ECF83D9-6B67-4165-A588-8B0B40CB0EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="697" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="697" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicative Elements" sheetId="4" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="275">
   <si>
     <t>Method</t>
   </si>
@@ -940,9 +940,6 @@
   </si>
   <si>
     <t>Sr (ppm)</t>
-  </si>
-  <si>
-    <t>Carpathian</t>
   </si>
   <si>
     <t>Göllü Dag</t>
@@ -5919,7 +5916,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -6201,15 +6198,15 @@
         <v>61</v>
       </c>
       <c r="I20" t="s">
+        <v>273</v>
+      </c>
+      <c r="J20" t="s">
         <v>274</v>
-      </c>
-      <c r="J20" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B21">
         <v>298</v>
@@ -6241,7 +6238,7 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B22">
         <v>312</v>
@@ -6273,7 +6270,7 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B23">
         <v>229</v>
@@ -6305,7 +6302,7 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B24">
         <v>307</v>
@@ -6337,7 +6334,7 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B25">
         <v>237</v>
@@ -6369,7 +6366,7 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B26">
         <v>417</v>
@@ -6401,7 +6398,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B27">
         <v>573</v>
@@ -7103,7 +7100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>73</v>
       </c>
@@ -7135,7 +7132,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>73</v>
       </c>
@@ -7167,7 +7164,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>73</v>
       </c>
@@ -7199,7 +7196,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>29</v>
       </c>
@@ -7231,7 +7228,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>29</v>
       </c>
@@ -7263,7 +7260,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>29</v>
       </c>
@@ -7295,7 +7292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>29</v>
       </c>
@@ -7327,7 +7324,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>29</v>
       </c>
@@ -7359,541 +7356,487 @@
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>272</v>
+        <v>17</v>
       </c>
       <c r="B57">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="C57">
-        <v>232</v>
+        <v>300</v>
       </c>
       <c r="D57">
+        <v>5536</v>
+      </c>
+      <c r="E57">
+        <v>23</v>
+      </c>
+      <c r="F57">
+        <v>155</v>
+      </c>
+      <c r="G57">
+        <v>73</v>
+      </c>
+      <c r="H57">
+        <v>69</v>
+      </c>
+      <c r="I57">
+        <v>359</v>
+      </c>
+      <c r="J57">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>17</v>
+      </c>
+      <c r="B58">
+        <v>188</v>
+      </c>
+      <c r="C58">
+        <v>282</v>
+      </c>
+      <c r="D58">
+        <v>5404</v>
+      </c>
+      <c r="E58">
+        <v>21</v>
+      </c>
+      <c r="F58">
+        <v>154</v>
+      </c>
+      <c r="G58">
+        <v>76</v>
+      </c>
+      <c r="H58">
+        <v>69</v>
+      </c>
+      <c r="I58">
+        <v>326</v>
+      </c>
+      <c r="J58">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>17</v>
+      </c>
+      <c r="B59">
+        <v>223</v>
+      </c>
+      <c r="C59">
+        <v>305</v>
+      </c>
+      <c r="D59">
+        <v>5261</v>
+      </c>
+      <c r="E59">
+        <v>23</v>
+      </c>
+      <c r="F59">
+        <v>163</v>
+      </c>
+      <c r="G59">
+        <v>77</v>
+      </c>
+      <c r="H59">
+        <v>63</v>
+      </c>
+      <c r="I59">
+        <v>280</v>
+      </c>
+      <c r="J59">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>17</v>
+      </c>
+      <c r="B60">
+        <v>231</v>
+      </c>
+      <c r="C60">
+        <v>291</v>
+      </c>
+      <c r="D60">
+        <v>4768</v>
+      </c>
+      <c r="E60">
+        <v>22</v>
+      </c>
+      <c r="F60">
+        <v>156</v>
+      </c>
+      <c r="G60">
+        <v>65</v>
+      </c>
+      <c r="H60">
+        <v>62</v>
+      </c>
+      <c r="I60">
+        <v>420</v>
+      </c>
+      <c r="J60">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>17</v>
+      </c>
+      <c r="B61">
+        <v>231</v>
+      </c>
+      <c r="C61">
+        <v>326</v>
+      </c>
+      <c r="D61">
+        <v>5187</v>
+      </c>
+      <c r="E61">
+        <v>22</v>
+      </c>
+      <c r="F61">
+        <v>172</v>
+      </c>
+      <c r="G61">
+        <v>73</v>
+      </c>
+      <c r="H61">
+        <v>68</v>
+      </c>
+      <c r="I61">
+        <v>305</v>
+      </c>
+      <c r="J61">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>17</v>
+      </c>
+      <c r="B62">
+        <v>229</v>
+      </c>
+      <c r="C62">
+        <v>308</v>
+      </c>
+      <c r="D62">
+        <v>5456</v>
+      </c>
+      <c r="E62">
+        <v>22</v>
+      </c>
+      <c r="F62">
+        <v>168</v>
+      </c>
+      <c r="G62">
+        <v>75</v>
+      </c>
+      <c r="H62">
+        <v>74</v>
+      </c>
+      <c r="I62">
+        <v>351</v>
+      </c>
+      <c r="J62">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63">
+        <v>170</v>
+      </c>
+      <c r="C63">
+        <v>340</v>
+      </c>
+      <c r="D63">
+        <v>5483</v>
+      </c>
+      <c r="E63">
+        <v>20</v>
+      </c>
+      <c r="F63">
+        <v>173</v>
+      </c>
+      <c r="G63">
+        <v>64</v>
+      </c>
+      <c r="H63">
+        <v>67</v>
+      </c>
+      <c r="I63">
+        <v>307</v>
+      </c>
+      <c r="J63">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64">
+        <v>1701</v>
+      </c>
+      <c r="C64">
+        <v>421</v>
+      </c>
+      <c r="D64">
+        <v>11671</v>
+      </c>
+      <c r="E64">
+        <v>46</v>
+      </c>
+      <c r="F64">
+        <v>174</v>
+      </c>
+      <c r="G64">
+        <v>71</v>
+      </c>
+      <c r="H64">
+        <v>128</v>
+      </c>
+      <c r="I64">
+        <v>367</v>
+      </c>
+      <c r="J64">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>18</v>
+      </c>
+      <c r="B65">
+        <v>364</v>
+      </c>
+      <c r="C65">
+        <v>258</v>
+      </c>
+      <c r="D65">
+        <v>7335</v>
+      </c>
+      <c r="E65">
+        <v>46</v>
+      </c>
+      <c r="F65">
+        <v>185</v>
+      </c>
+      <c r="G65">
+        <v>75</v>
+      </c>
+      <c r="H65">
+        <v>122</v>
+      </c>
+      <c r="I65">
+        <v>408</v>
+      </c>
+      <c r="J65">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>18</v>
+      </c>
+      <c r="B66">
+        <v>682</v>
+      </c>
+      <c r="C66">
         <v>300</v>
       </c>
-      <c r="E57">
-        <v>5536</v>
-      </c>
-      <c r="F57">
-        <v>23</v>
-      </c>
-      <c r="G57">
-        <v>155</v>
-      </c>
-      <c r="H57">
+      <c r="D66">
+        <v>7315</v>
+      </c>
+      <c r="E66">
+        <v>32</v>
+      </c>
+      <c r="F66">
+        <v>164</v>
+      </c>
+      <c r="G66">
+        <v>70</v>
+      </c>
+      <c r="H66">
+        <v>129</v>
+      </c>
+      <c r="I66">
+        <v>416</v>
+      </c>
+      <c r="J66">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67">
+        <v>327</v>
+      </c>
+      <c r="C67">
+        <v>289</v>
+      </c>
+      <c r="D67">
+        <v>7512</v>
+      </c>
+      <c r="E67">
+        <v>37</v>
+      </c>
+      <c r="F67">
+        <v>181</v>
+      </c>
+      <c r="G67">
+        <v>71</v>
+      </c>
+      <c r="H67">
+        <v>126</v>
+      </c>
+      <c r="I67">
+        <v>459</v>
+      </c>
+      <c r="J67">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68">
+        <v>326</v>
+      </c>
+      <c r="C68">
+        <v>286</v>
+      </c>
+      <c r="D68">
+        <v>7052</v>
+      </c>
+      <c r="E68">
+        <v>35</v>
+      </c>
+      <c r="F68">
+        <v>165</v>
+      </c>
+      <c r="G68">
+        <v>72</v>
+      </c>
+      <c r="H68">
+        <v>118</v>
+      </c>
+      <c r="I68">
+        <v>407</v>
+      </c>
+      <c r="J68">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>18</v>
+      </c>
+      <c r="B69">
+        <v>331</v>
+      </c>
+      <c r="C69">
+        <v>296</v>
+      </c>
+      <c r="D69">
+        <v>7108</v>
+      </c>
+      <c r="E69">
+        <v>36</v>
+      </c>
+      <c r="F69">
+        <v>173</v>
+      </c>
+      <c r="G69">
+        <v>72</v>
+      </c>
+      <c r="H69">
+        <v>123</v>
+      </c>
+      <c r="I69">
+        <v>461</v>
+      </c>
+      <c r="J69">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>18</v>
+      </c>
+      <c r="B70">
+        <v>2356</v>
+      </c>
+      <c r="C70">
+        <v>278</v>
+      </c>
+      <c r="D70">
+        <v>12551</v>
+      </c>
+      <c r="E70">
+        <v>43</v>
+      </c>
+      <c r="F70">
+        <v>176</v>
+      </c>
+      <c r="G70">
         <v>73</v>
       </c>
-      <c r="I57">
-        <v>69</v>
-      </c>
-      <c r="J57">
-        <v>359</v>
-      </c>
-      <c r="K57">
+      <c r="H70">
+        <v>128</v>
+      </c>
+      <c r="I70">
+        <v>385</v>
+      </c>
+      <c r="J70">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>18</v>
+      </c>
+      <c r="B71">
+        <v>2032</v>
+      </c>
+      <c r="C71">
+        <v>292</v>
+      </c>
+      <c r="D71">
+        <v>11361</v>
+      </c>
+      <c r="E71">
+        <v>38</v>
+      </c>
+      <c r="F71">
+        <v>174</v>
+      </c>
+      <c r="G71">
+        <v>74</v>
+      </c>
+      <c r="H71">
+        <v>133</v>
+      </c>
+      <c r="I71">
+        <v>572</v>
+      </c>
+      <c r="J71">
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>272</v>
-      </c>
-      <c r="B58">
-        <v>1</v>
-      </c>
-      <c r="C58">
-        <v>188</v>
-      </c>
-      <c r="D58">
-        <v>282</v>
-      </c>
-      <c r="E58">
-        <v>5404</v>
-      </c>
-      <c r="F58">
-        <v>21</v>
-      </c>
-      <c r="G58">
-        <v>154</v>
-      </c>
-      <c r="H58">
-        <v>76</v>
-      </c>
-      <c r="I58">
-        <v>69</v>
-      </c>
-      <c r="J58">
-        <v>326</v>
-      </c>
-      <c r="K58">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>272</v>
-      </c>
-      <c r="B59">
-        <v>1</v>
-      </c>
-      <c r="C59">
-        <v>223</v>
-      </c>
-      <c r="D59">
-        <v>305</v>
-      </c>
-      <c r="E59">
-        <v>5261</v>
-      </c>
-      <c r="F59">
-        <v>23</v>
-      </c>
-      <c r="G59">
-        <v>163</v>
-      </c>
-      <c r="H59">
-        <v>77</v>
-      </c>
-      <c r="I59">
-        <v>63</v>
-      </c>
-      <c r="J59">
-        <v>280</v>
-      </c>
-      <c r="K59">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>272</v>
-      </c>
-      <c r="B60">
-        <v>1</v>
-      </c>
-      <c r="C60">
-        <v>231</v>
-      </c>
-      <c r="D60">
-        <v>291</v>
-      </c>
-      <c r="E60">
-        <v>4768</v>
-      </c>
-      <c r="F60">
-        <v>22</v>
-      </c>
-      <c r="G60">
-        <v>156</v>
-      </c>
-      <c r="H60">
-        <v>65</v>
-      </c>
-      <c r="I60">
-        <v>62</v>
-      </c>
-      <c r="J60">
-        <v>420</v>
-      </c>
-      <c r="K60">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>272</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61">
-        <v>231</v>
-      </c>
-      <c r="D61">
-        <v>326</v>
-      </c>
-      <c r="E61">
-        <v>5187</v>
-      </c>
-      <c r="F61">
-        <v>22</v>
-      </c>
-      <c r="G61">
-        <v>172</v>
-      </c>
-      <c r="H61">
-        <v>73</v>
-      </c>
-      <c r="I61">
-        <v>68</v>
-      </c>
-      <c r="J61">
-        <v>305</v>
-      </c>
-      <c r="K61">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>272</v>
-      </c>
-      <c r="B62">
-        <v>1</v>
-      </c>
-      <c r="C62">
-        <v>229</v>
-      </c>
-      <c r="D62">
-        <v>308</v>
-      </c>
-      <c r="E62">
-        <v>5456</v>
-      </c>
-      <c r="F62">
-        <v>22</v>
-      </c>
-      <c r="G62">
-        <v>168</v>
-      </c>
-      <c r="H62">
-        <v>75</v>
-      </c>
-      <c r="I62">
-        <v>74</v>
-      </c>
-      <c r="J62">
-        <v>351</v>
-      </c>
-      <c r="K62">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>272</v>
-      </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="C63">
-        <v>170</v>
-      </c>
-      <c r="D63">
-        <v>340</v>
-      </c>
-      <c r="E63">
-        <v>5483</v>
-      </c>
-      <c r="F63">
-        <v>20</v>
-      </c>
-      <c r="G63">
-        <v>173</v>
-      </c>
-      <c r="H63">
-        <v>64</v>
-      </c>
-      <c r="I63">
-        <v>67</v>
-      </c>
-      <c r="J63">
-        <v>307</v>
-      </c>
-      <c r="K63">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>272</v>
-      </c>
-      <c r="B64">
-        <v>2</v>
-      </c>
-      <c r="C64">
-        <v>1701</v>
-      </c>
-      <c r="D64">
-        <v>421</v>
-      </c>
-      <c r="E64">
-        <v>11</v>
-      </c>
-      <c r="F64">
-        <v>671</v>
-      </c>
-      <c r="G64">
-        <v>46</v>
-      </c>
-      <c r="H64">
-        <v>174</v>
-      </c>
-      <c r="I64">
-        <v>71</v>
-      </c>
-      <c r="J64">
-        <v>128</v>
-      </c>
-      <c r="K64">
-        <v>367</v>
-      </c>
-      <c r="L64">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>272</v>
-      </c>
-      <c r="B65">
-        <v>2</v>
-      </c>
-      <c r="C65">
-        <v>364</v>
-      </c>
-      <c r="D65">
-        <v>258</v>
-      </c>
-      <c r="E65">
-        <v>7335</v>
-      </c>
-      <c r="F65">
-        <v>46</v>
-      </c>
-      <c r="G65">
-        <v>185</v>
-      </c>
-      <c r="H65">
-        <v>75</v>
-      </c>
-      <c r="I65">
-        <v>122</v>
-      </c>
-      <c r="J65">
-        <v>408</v>
-      </c>
-      <c r="K65">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>272</v>
-      </c>
-      <c r="B66">
-        <v>2</v>
-      </c>
-      <c r="C66">
-        <v>682</v>
-      </c>
-      <c r="D66">
-        <v>300</v>
-      </c>
-      <c r="E66">
-        <v>7315</v>
-      </c>
-      <c r="F66">
-        <v>32</v>
-      </c>
-      <c r="G66">
-        <v>164</v>
-      </c>
-      <c r="H66">
-        <v>70</v>
-      </c>
-      <c r="I66">
-        <v>129</v>
-      </c>
-      <c r="J66">
-        <v>416</v>
-      </c>
-      <c r="K66">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>272</v>
-      </c>
-      <c r="B67">
-        <v>2</v>
-      </c>
-      <c r="C67">
-        <v>327</v>
-      </c>
-      <c r="D67">
-        <v>289</v>
-      </c>
-      <c r="E67">
-        <v>7512</v>
-      </c>
-      <c r="F67">
-        <v>37</v>
-      </c>
-      <c r="G67">
-        <v>181</v>
-      </c>
-      <c r="H67">
-        <v>71</v>
-      </c>
-      <c r="I67">
-        <v>126</v>
-      </c>
-      <c r="J67">
-        <v>459</v>
-      </c>
-      <c r="K67">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>272</v>
-      </c>
-      <c r="B68">
-        <v>2</v>
-      </c>
-      <c r="C68">
-        <v>326</v>
-      </c>
-      <c r="D68">
-        <v>286</v>
-      </c>
-      <c r="E68">
-        <v>7052</v>
-      </c>
-      <c r="F68">
-        <v>35</v>
-      </c>
-      <c r="G68">
-        <v>165</v>
-      </c>
-      <c r="H68">
-        <v>72</v>
-      </c>
-      <c r="I68">
-        <v>118</v>
-      </c>
-      <c r="J68">
-        <v>407</v>
-      </c>
-      <c r="K68">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>272</v>
-      </c>
-      <c r="B69">
-        <v>2</v>
-      </c>
-      <c r="C69">
-        <v>331</v>
-      </c>
-      <c r="D69">
-        <v>296</v>
-      </c>
-      <c r="E69">
-        <v>7108</v>
-      </c>
-      <c r="F69">
-        <v>36</v>
-      </c>
-      <c r="G69">
-        <v>173</v>
-      </c>
-      <c r="H69">
-        <v>72</v>
-      </c>
-      <c r="I69">
-        <v>123</v>
-      </c>
-      <c r="J69">
-        <v>461</v>
-      </c>
-      <c r="K69">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>272</v>
-      </c>
-      <c r="B70">
-        <v>2</v>
-      </c>
-      <c r="C70">
-        <v>2356</v>
-      </c>
-      <c r="D70">
-        <v>278</v>
-      </c>
-      <c r="E70">
-        <v>12</v>
-      </c>
-      <c r="F70">
-        <v>551</v>
-      </c>
-      <c r="G70">
-        <v>43</v>
-      </c>
-      <c r="H70">
-        <v>176</v>
-      </c>
-      <c r="I70">
-        <v>73</v>
-      </c>
-      <c r="J70">
-        <v>128</v>
-      </c>
-      <c r="K70">
-        <v>385</v>
-      </c>
-      <c r="L70">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>272</v>
-      </c>
-      <c r="B71">
-        <v>2</v>
-      </c>
-      <c r="C71">
-        <v>2032</v>
-      </c>
-      <c r="D71">
-        <v>292</v>
-      </c>
-      <c r="E71">
-        <v>11</v>
-      </c>
-      <c r="F71">
-        <v>361</v>
-      </c>
-      <c r="G71">
-        <v>38</v>
-      </c>
-      <c r="H71">
-        <v>174</v>
-      </c>
-      <c r="I71">
-        <v>74</v>
-      </c>
-      <c r="J71">
-        <v>133</v>
-      </c>
-      <c r="K71">
-        <v>572</v>
-      </c>
-      <c r="L71">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>16</v>
       </c>

</xml_diff>